<commit_message>
Sync canonical feedback composition
</commit_message>
<xml_diff>
--- a/hotel_pl_normalizer/data/output_template.xlsx
+++ b/hotel_pl_normalizer/data/output_template.xlsx
@@ -1371,283 +1371,283 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="6">
-    <x:numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <x:numFmt numFmtId="164" formatCode="_(#,##0_);[Red]_(\(#,##0\);_(\ \-\ _);@_)"/>
-    <x:numFmt numFmtId="165" formatCode="0.0_)%;\(0.0\)%;0.0%_);@_)_%"/>
-    <x:numFmt numFmtId="166" formatCode="_(#,##0.00_);[Red]_(\(#,##0.00\);_(\ \-\ _);@_)"/>
-    <x:numFmt numFmtId="167" formatCode="0.0_)%;\(0.0\)%;0.0_)%;@_)_%"/>
-    <x:numFmt numFmtId="168" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* \-\ _);@_)"/>
-  </x:numFmts>
-  <x:fonts count="17">
-    <x:font>
-      <x:sz val="11"/>
-      <x:color theme="1"/>
-      <x:name val="Aptos Narrow"/>
-    </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color theme="1"/>
-      <x:name val="Aptos Narrow"/>
-    </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color theme="1"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color indexed="9"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FFFFFFFF"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:sz val="9"/>
-      <x:color theme="1"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:sz val="9"/>
-      <x:color theme="1"/>
-      <x:name val="Aptos Narrow"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="9"/>
-      <x:color indexed="9"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="9"/>
-      <x:color theme="1"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:sz val="9"/>
-      <x:color theme="1"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:sz val="9"/>
-      <x:color indexed="12"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="9"/>
-      <x:color theme="1"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:sz val="9"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:sz val="9"/>
-      <x:color indexed="12"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:i/>
-      <x:sz val="9"/>
-      <x:color theme="1"/>
-      <x:name val="Calibri"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="6">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF39617A"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF39617A"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFEEECE1"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFFFFF"/>
-      </x:patternFill>
-    </x:fill>
-  </x:fills>
-  <x:borders count="5">
-    <x:border/>
-    <x:border>
-      <x:top style="thin">
-        <x:color indexed="64"/>
-      </x:top>
-    </x:border>
-    <x:border>
-      <x:bottom style="thin">
-        <x:color indexed="64"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
-      <x:bottom style="hair">
-        <x:color indexed="64"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color indexed="64"/>
-      </x:left>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="2">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <x:xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
-  </x:cellStyleXfs>
-  <x:cellXfs count="57">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="left" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <x:xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="right"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <x:xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <x:xf numFmtId="168" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <x:xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="centerContinuous"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="38" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <x:xf numFmtId="38" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="38" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="40" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="38" fontId="14" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="38" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <x:xf numFmtId="40" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="38" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="38" fontId="11" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="38" fontId="15" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="167" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <x:xf numFmtId="38" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <x:alignment horizontal="left"/>
-    </x:xf>
-    <x:xf numFmtId="38" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="38" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="167" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <x:xf numFmtId="40" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <x:xf numFmtId="38" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-  </x:cellXfs>
-  <x:cellStyles count="2">
-    <x:cellStyle name="Comma" xfId="1"/>
-    <x:cellStyle name="Normal" xfId="0"/>
-  </x:cellStyles>
-  <x:dxfs count="2">
-    <x:dxf>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFEEECE1"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFEEECE1"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-  </x:dxfs>
-</x:styleSheet>
+<ns0:styleSheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:numFmts count="6">
+    <ns0:numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <ns0:numFmt numFmtId="164" formatCode="_(#,##0_);[Red]_(\(#,##0\);_(\ \-\ _);@_)"/>
+    <ns0:numFmt numFmtId="165" formatCode="0.0_)%;\(0.0\)%;0.0%_);@_)_%"/>
+    <ns0:numFmt numFmtId="166" formatCode="_(#,##0.00_);[Red]_(\(#,##0.00\);_(\ \-\ _);@_)"/>
+    <ns0:numFmt numFmtId="167" formatCode="0.0_)%;\(0.0\)%;0.0_)%;@_)_%"/>
+    <ns0:numFmt numFmtId="168" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* \-\ _);@_)"/>
+  </ns0:numFmts>
+  <ns0:fonts count="17">
+    <ns0:font>
+      <ns0:sz val="11"/>
+      <ns0:color theme="1"/>
+      <ns0:name val="Aptos Narrow"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="11"/>
+      <ns0:color theme="1"/>
+      <ns0:name val="Aptos Narrow"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="11"/>
+      <ns0:color theme="1"/>
+      <ns0:name val="Calibri"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="11"/>
+      <ns0:color indexed="9"/>
+      <ns0:name val="Calibri"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="11"/>
+      <ns0:color rgb="FFFFFFFF"/>
+      <ns0:name val="Calibri"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="11"/>
+      <ns0:name val="Calibri"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="11"/>
+      <ns0:name val="Calibri"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="9"/>
+      <ns0:color theme="1"/>
+      <ns0:name val="Calibri"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="9"/>
+      <ns0:color theme="1"/>
+      <ns0:name val="Aptos Narrow"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="9"/>
+      <ns0:color indexed="9"/>
+      <ns0:name val="Calibri"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="9"/>
+      <ns0:color theme="1"/>
+      <ns0:name val="Calibri"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="9"/>
+      <ns0:color theme="1"/>
+      <ns0:name val="Calibri"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="9"/>
+      <ns0:color indexed="12"/>
+      <ns0:name val="Calibri"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:b/>
+      <ns0:sz val="9"/>
+      <ns0:color theme="1"/>
+      <ns0:name val="Calibri"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="9"/>
+      <ns0:name val="Calibri"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="9"/>
+      <ns0:color indexed="12"/>
+      <ns0:name val="Calibri"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:i/>
+      <ns0:sz val="9"/>
+      <ns0:color theme="1"/>
+      <ns0:name val="Calibri"/>
+    </ns0:font>
+  </ns0:fonts>
+  <ns0:fills count="6">
+    <ns0:fill>
+      <ns0:patternFill patternType="none"/>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="gray125"/>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FF39617A"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FF39617A"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFEEECE1"/>
+      </ns0:patternFill>
+    </ns0:fill>
+    <ns0:fill>
+      <ns0:patternFill patternType="solid">
+        <ns0:fgColor rgb="FFFFFFFF"/>
+      </ns0:patternFill>
+    </ns0:fill>
+  </ns0:fills>
+  <ns0:borders count="5">
+    <ns0:border/>
+    <ns0:border>
+      <ns0:top style="thin">
+        <ns0:color indexed="64"/>
+      </ns0:top>
+    </ns0:border>
+    <ns0:border>
+      <ns0:bottom style="thin">
+        <ns0:color indexed="64"/>
+      </ns0:bottom>
+    </ns0:border>
+    <ns0:border>
+      <ns0:bottom style="hair">
+        <ns0:color indexed="64"/>
+      </ns0:bottom>
+    </ns0:border>
+    <ns0:border>
+      <ns0:left style="thin">
+        <ns0:color indexed="64"/>
+      </ns0:left>
+    </ns0:border>
+  </ns0:borders>
+  <ns0:cellStyleXfs count="2">
+    <ns0:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <ns0:xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
+  </ns0:cellStyleXfs>
+  <ns0:cellXfs count="57">
+    <ns0:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <ns0:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <ns0:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <ns0:alignment horizontal="left"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <ns0:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <ns0:alignment wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <ns0:xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <ns0:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <ns0:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <ns0:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <ns0:alignment horizontal="left"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <ns0:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <ns0:xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <ns0:alignment horizontal="left"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <ns0:xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <ns0:alignment horizontal="right"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <ns0:xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <ns0:xf numFmtId="168" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <ns0:xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <ns0:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <ns0:alignment horizontal="centerContinuous"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <ns0:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" indent="2"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="38" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <ns0:xf numFmtId="38" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <ns0:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" indent="5"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" indent="5"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <ns0:alignment horizontal="left"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="38" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <ns0:xf numFmtId="40" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <ns0:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" indent="8"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="38" fontId="14" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <ns0:xf numFmtId="38" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <ns0:xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <ns0:xf numFmtId="40" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <ns0:xf numFmtId="38" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <ns0:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" indent="3"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" indent="4"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="38" fontId="11" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <ns0:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" indent="7"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="38" fontId="15" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <ns0:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" indent="6"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="167" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <ns0:xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <ns0:xf numFmtId="38" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <ns0:xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <ns0:alignment horizontal="left" indent="8"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="38" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <ns0:xf numFmtId="38" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <ns0:xf numFmtId="167" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <ns0:xf numFmtId="40" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <ns0:xf numFmtId="38" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <ns0:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <ns0:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+  </ns0:cellXfs>
+  <ns0:cellStyles count="2">
+    <ns0:cellStyle name="Comma" xfId="1"/>
+    <ns0:cellStyle name="Normal" xfId="0"/>
+  </ns0:cellStyles>
+  <ns0:dxfs count="2">
+    <ns0:dxf>
+      <ns0:fill>
+        <ns0:patternFill>
+          <ns0:bgColor rgb="FFEEECE1"/>
+        </ns0:patternFill>
+      </ns0:fill>
+    </ns0:dxf>
+    <ns0:dxf>
+      <ns0:fill>
+        <ns0:patternFill patternType="solid">
+          <ns0:bgColor rgb="FFEEECE1"/>
+        </ns0:patternFill>
+      </ns0:fill>
+    </ns0:dxf>
+  </ns0:dxfs>
+</ns0:styleSheet>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>